<commit_message>
Tablero HTML: rediseño visual con marca HDI y tema claro/oscuro
- Nueva paleta de marca (verde HDI), soporte de tema oscuro y logo
  embebido en el notebook y en el HTML generado (reports/).
- Se agrega export .aspx del tablero y el logo HDI_Seguros.png.
- Se archivan versiones previas del dashboard Power BI en
  reportes_anteriores/ (pbix + pdf) como respaldo histórico.
- Ajustes menores en el catálogo de reglas (docs/*.xlsx).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KPIs - REGLAS CALIDAD CDP Primas.xlsx
+++ b/docs/KPIs - REGLAS CALIDAD CDP Primas.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hdiseguroscom-my.sharepoint.com/personal/juan_rojas_outsourcing_hdiseguros_com_co/Documents/Documentos/HDI/Data QA/Sprint 4/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hdiseguroscom-my.sharepoint.com/personal/wilson_jerez_hdiseguros_com_co/Documents/Documentos/hdi-primas-data-quality/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="597" documentId="8_{D2055801-B4CA-4B50-B828-52150F4FC6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{121D7DC3-8229-4DC2-B70A-A15F9E1886A8}"/>
+  <xr:revisionPtr revIDLastSave="611" documentId="8_{D2055801-B4CA-4B50-B828-52150F4FC6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58C84EF1-9A16-4CD2-B1C1-206C05154911}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{BFEF58F7-4A30-46F0-8EB3-9D58F8779212}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BFEF58F7-4A30-46F0-8EB3-9D58F8779212}"/>
   </bookViews>
   <sheets>
     <sheet name="Reglas KPIs Calidad" sheetId="1" r:id="rId1"/>
     <sheet name="Filtros a tener en cuenta" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reglas KPIs Calidad'!$A$2:$N$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reglas KPIs Calidad'!$A$1:$N$27</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -4303,10 +4303,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
@@ -4325,7 +4323,8 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4701,11 +4700,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F6143CF-73B8-4D5B-AC7B-57720CE1FA6E}">
-  <dimension ref="A1:R28"/>
+  <dimension ref="A1:R27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="45.1796875" customWidth="1"/>
     <col min="3" max="3" width="32.26953125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.36328125" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="41.81640625" bestFit="1" customWidth="1"/>
@@ -4724,1133 +4723,1116 @@
     <col min="18" max="18" width="40.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="I1">
+    <row r="1" spans="1:18" s="10" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="J1">
+      <c r="D1" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="K1">
-        <v>3</v>
-      </c>
-      <c r="L1">
-        <v>2</v>
-      </c>
-      <c r="M1">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="O1" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="P1" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q1" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="R1" s="10" t="s">
+        <v>95</v>
+      </c>
     </row>
-    <row r="2" spans="1:18" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>95</v>
-      </c>
+    <row r="2" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="J2" s="3"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
     </row>
-    <row r="3" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:18" ht="116" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="E3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="O3" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="1"/>
+    </row>
+    <row r="4" spans="1:18" ht="232" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3" t="s">
+      <c r="G4" s="1"/>
+      <c r="H4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="J3" s="5"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-      <c r="O3" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
+      <c r="I4" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J4" s="1"/>
+      <c r="K4" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="R4" s="6" t="s">
+        <v>96</v>
+      </c>
     </row>
-    <row r="4" spans="1:18" ht="116" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B5" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C5" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="3" t="s">
+      <c r="E5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" s="3" t="s">
+      <c r="G5" s="1"/>
+      <c r="H5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="1"/>
+    </row>
+    <row r="6" spans="1:18" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J4" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="O4" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="P4" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="5" t="s">
+        <v>97</v>
+      </c>
     </row>
-    <row r="5" spans="1:18" ht="232" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B7" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C7" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" s="3" t="s">
+      <c r="E7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="1"/>
+    </row>
+    <row r="8" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3" t="s">
+      <c r="G8" s="1"/>
+      <c r="H8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I8" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J5" s="3"/>
-      <c r="K5" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="L5" s="5" t="s">
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="R5" s="8" t="s">
-        <v>96</v>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="5" t="s">
+        <v>98</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+    <row r="9" spans="1:18" ht="26" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B9" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C9" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="3" t="s">
+      <c r="E9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3" t="s">
+      <c r="G9" s="1"/>
+      <c r="H9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
+      <c r="I9" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="1"/>
+      <c r="R9" s="1"/>
     </row>
-    <row r="7" spans="1:18" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+    <row r="10" spans="1:18" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B10" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C10" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3" t="s">
+      <c r="E10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I10" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="7" t="s">
-        <v>97</v>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="1"/>
+      <c r="R10" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
+    <row r="11" spans="1:18" ht="58" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B11" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C11" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D11" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" s="3" t="s">
+      <c r="E11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3" t="s">
+      <c r="G11" s="1"/>
+      <c r="H11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="3"/>
-      <c r="P8" s="3"/>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="3"/>
+      <c r="I11" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="1"/>
+      <c r="R11" s="5" t="s">
+        <v>100</v>
+      </c>
     </row>
-    <row r="9" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
+    <row r="12" spans="1:18" ht="116" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B12" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C12" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3" t="s">
+      <c r="E12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="I12" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="P9" s="3"/>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="7" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" ht="26" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="P10" s="3"/>
-      <c r="Q10" s="3"/>
-      <c r="R10" s="3"/>
-    </row>
-    <row r="11" spans="1:18" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="P11" s="3"/>
-      <c r="Q11" s="3"/>
-      <c r="R11" s="7" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="58" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3" t="s">
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
-      <c r="O12" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="P12" s="3"/>
-      <c r="Q12" s="3"/>
-      <c r="R12" s="7" t="s">
-        <v>100</v>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="P12" s="1"/>
+      <c r="Q12" s="1"/>
+      <c r="R12" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="116" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F13" s="3" t="s">
+      <c r="E13" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3" t="s">
+      <c r="G13" s="1"/>
+      <c r="H13" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="I13" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3" t="s">
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="O13" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="P13" s="3"/>
-      <c r="Q13" s="3"/>
-      <c r="R13" s="7" t="s">
-        <v>101</v>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="P13" s="1"/>
+      <c r="Q13" s="1"/>
+      <c r="R13" s="5" t="s">
+        <v>102</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="116" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:18" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F14" s="3" t="s">
+      <c r="E14" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3" t="s">
+      <c r="G14" s="1"/>
+      <c r="H14" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="I14" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3" t="s">
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
-      <c r="O14" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="P14" s="3"/>
-      <c r="Q14" s="3"/>
-      <c r="R14" s="7" t="s">
-        <v>102</v>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1"/>
+      <c r="R14" s="5" t="s">
+        <v>103</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F15" s="3" t="s">
+      <c r="E15" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="P15" s="1"/>
+      <c r="Q15" s="1"/>
+      <c r="R15" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
+      <c r="R16" s="1"/>
+    </row>
+    <row r="17" spans="1:18" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3" t="s">
+      <c r="G17" s="1"/>
+      <c r="H17" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I15" s="3" t="s">
+      <c r="I17" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="P15" s="3"/>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="7" t="s">
-        <v>103</v>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="P17" s="1"/>
+      <c r="Q17" s="1"/>
+      <c r="R17" s="5" t="s">
+        <v>105</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
+    <row r="18" spans="1:18" ht="52" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B18" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C18" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D18" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E16" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F16" s="3" t="s">
+      <c r="E18" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3" t="s">
+      <c r="G18" s="1"/>
+      <c r="H18" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="I18" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
-      <c r="O16" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="P16" s="3"/>
-      <c r="Q16" s="3"/>
-      <c r="R16" s="7" t="s">
-        <v>104</v>
-      </c>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="P18" s="1"/>
+      <c r="Q18" s="1"/>
+      <c r="R18" s="1"/>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A17" s="3" t="s">
+    <row r="19" spans="1:18" ht="217.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B19" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C19" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D19" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F17" s="3" t="s">
+      <c r="E19" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3" t="s">
+      <c r="G19" s="1"/>
+      <c r="H19" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
-      <c r="O17" s="3"/>
-      <c r="P17" s="3"/>
-      <c r="Q17" s="3"/>
-      <c r="R17" s="3"/>
+      <c r="I19" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J19" s="1"/>
+      <c r="K19" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="P19" s="1"/>
+      <c r="Q19" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="R19" s="6" t="s">
+        <v>106</v>
+      </c>
     </row>
-    <row r="18" spans="1:18" ht="130.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="3" t="s">
+    <row r="20" spans="1:18" ht="52" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B20" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C20" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D20" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E18" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F18" s="3" t="s">
+      <c r="E20" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="N20" s="1"/>
+      <c r="O20" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="P20" s="1"/>
+      <c r="Q20" s="1"/>
+      <c r="R20" s="1"/>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="N21" s="1"/>
+      <c r="O21" s="1"/>
+      <c r="P21" s="1"/>
+      <c r="Q21" s="1"/>
+      <c r="R21" s="1"/>
+    </row>
+    <row r="22" spans="1:18" ht="52" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="N22" s="1"/>
+      <c r="O22" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="P22" s="1"/>
+      <c r="Q22" s="1"/>
+      <c r="R22" s="1"/>
+    </row>
+    <row r="23" spans="1:18" ht="246.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="R23" s="1"/>
+    </row>
+    <row r="24" spans="1:18" ht="232" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3" t="s">
+      <c r="G24" s="1"/>
+      <c r="H24" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I18" s="3" t="s">
+      <c r="I24" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="1"/>
+      <c r="R24" s="1"/>
+    </row>
+    <row r="25" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="M18" s="3"/>
-      <c r="N18" s="3"/>
-      <c r="O18" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="P18" s="3"/>
-      <c r="Q18" s="3"/>
-      <c r="R18" s="7" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18" ht="52" x14ac:dyDescent="0.35">
-      <c r="A19" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="P19" s="3"/>
-      <c r="Q19" s="3"/>
-      <c r="R19" s="3"/>
-    </row>
-    <row r="20" spans="1:18" ht="217.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="J20" s="3"/>
-      <c r="K20" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="L20" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="M20" s="3"/>
-      <c r="N20" s="3"/>
-      <c r="O20" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="P20" s="3"/>
-      <c r="Q20" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="R20" s="8" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="21" spans="1:18" ht="52" x14ac:dyDescent="0.35">
-      <c r="A21" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="3"/>
-      <c r="M21" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="N21" s="3"/>
-      <c r="O21" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="P21" s="3"/>
-      <c r="Q21" s="3"/>
-      <c r="R21" s="3"/>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A22" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
-      <c r="M22" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="N22" s="3"/>
-      <c r="O22" s="3"/>
-      <c r="P22" s="3"/>
-      <c r="Q22" s="3"/>
-      <c r="R22" s="3"/>
-    </row>
-    <row r="23" spans="1:18" ht="52" x14ac:dyDescent="0.35">
-      <c r="A23" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I23" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
-      <c r="L23" s="3"/>
-      <c r="M23" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="N23" s="3"/>
-      <c r="O23" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="P23" s="3"/>
-      <c r="Q23" s="3"/>
-      <c r="R23" s="3"/>
-    </row>
-    <row r="24" spans="1:18" ht="246.5" x14ac:dyDescent="0.35">
-      <c r="A24" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I24" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="J24" s="5"/>
-      <c r="K24" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="L24" s="3"/>
-      <c r="M24" s="3"/>
-      <c r="N24" s="3"/>
-      <c r="O24" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="P24" s="3"/>
-      <c r="Q24" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="R24" s="3"/>
-    </row>
-    <row r="25" spans="1:18" ht="232" x14ac:dyDescent="0.35">
-      <c r="A25" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G25" s="3"/>
-      <c r="H25" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I25" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="J25" s="3"/>
-      <c r="K25" s="3"/>
-      <c r="L25" s="3"/>
-      <c r="M25" s="3"/>
-      <c r="N25" s="3"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
       <c r="O25" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="P25" s="3"/>
-      <c r="Q25" s="3"/>
-      <c r="R25" s="3"/>
+        <v>86</v>
+      </c>
+      <c r="P25" s="1"/>
+      <c r="Q25" s="1"/>
+      <c r="R25" s="5" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="26" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E26" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F26" s="3" t="s">
+      <c r="E26" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3" t="s">
+      <c r="G26" s="1"/>
+      <c r="H26" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I26" s="3" t="s">
+      <c r="I26" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J26" s="3"/>
-      <c r="K26" s="3"/>
-      <c r="L26" s="5" t="s">
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="M26" s="3"/>
-      <c r="N26" s="3"/>
-      <c r="O26" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="P26" s="3"/>
-      <c r="Q26" s="3"/>
-      <c r="R26" s="7" t="s">
-        <v>107</v>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1"/>
+      <c r="R26" s="5" t="s">
+        <v>108</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A27" s="3" t="s">
+    <row r="27" spans="1:18" ht="52" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E27" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G27" s="3"/>
-      <c r="H27" s="3" t="s">
+      <c r="E27" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I27" s="3" t="s">
+      <c r="I27" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J27" s="3"/>
-      <c r="K27" s="3"/>
-      <c r="L27" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="M27" s="3"/>
-      <c r="N27" s="3"/>
-      <c r="O27" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="P27" s="3"/>
-      <c r="Q27" s="3"/>
-      <c r="R27" s="7" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="28" spans="1:18" ht="52" x14ac:dyDescent="0.35">
-      <c r="A28" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I28" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="J28" s="3"/>
-      <c r="K28" s="3"/>
-      <c r="L28" s="3"/>
-      <c r="M28" s="3" t="s">
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="N28" s="3"/>
-      <c r="O28" s="9" t="s">
+      <c r="N27" s="1"/>
+      <c r="O27" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="P28" s="3"/>
-      <c r="Q28" s="3"/>
-      <c r="R28" s="3"/>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1"/>
+      <c r="R27" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:N28" xr:uid="{9F6143CF-73B8-4D5B-AC7B-57720CE1FA6E}"/>
+  <autoFilter ref="A1:N27" xr:uid="{9F6143CF-73B8-4D5B-AC7B-57720CE1FA6E}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5860,74 +5842,74 @@
   <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="53.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="96.26953125" customWidth="1"/>
     <col min="2" max="2" width="35.54296875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="39.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="8" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="1" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="1" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="1" t="s">
         <v>117</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar cubo unificado, notebook runner, tablero HTML y catálogo de reglas
- sql/06_KPI_Cubo Unificado.sql y notebook runner: cambios recientes de lógica
- reports/tablero_calidad_primas.html: tablero regenerado
- docs: catálogo de reglas (xlsx/csv) actualizado
- Nuevo sql/00_ver.sql (consulta rápida de la vista fuente)
- .claude/settings.json versionado; settings.local.json ignorado

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KPIs - REGLAS CALIDAD CDP Primas.xlsx
+++ b/docs/KPIs - REGLAS CALIDAD CDP Primas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hdiseguroscom-my.sharepoint.com/personal/wilson_jerez_hdiseguros_com_co/Documents/Documentos/hdi-primas-data-quality/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="611" documentId="8_{D2055801-B4CA-4B50-B828-52150F4FC6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58C84EF1-9A16-4CD2-B1C1-206C05154911}"/>
+  <xr:revisionPtr revIDLastSave="627" documentId="8_{D2055801-B4CA-4B50-B828-52150F4FC6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{497711AE-5B7C-4332-A8B0-BEC81D7AEA04}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BFEF58F7-4A30-46F0-8EB3-9D58F8779212}"/>
   </bookViews>
@@ -4323,8 +4323,8 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4381,6 +4381,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4705,13 +4709,13 @@
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="45.1796875" customWidth="1"/>
-    <col min="3" max="3" width="32.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.6328125" customWidth="1"/>
     <col min="4" max="4" width="12.36328125" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="41.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.1796875" customWidth="1"/>
+    <col min="8" max="8" width="25.453125" customWidth="1"/>
+    <col min="9" max="9" width="32.7265625" customWidth="1"/>
     <col min="10" max="10" width="24.90625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="23.08984375" customWidth="1"/>
     <col min="12" max="12" width="24" bestFit="1" customWidth="1"/>

</xml_diff>